<commit_message>
feat: actualizar rubrica excel con lista de estudiantes de seccion martes
</commit_message>
<xml_diff>
--- a/docs/public/Rubrica_Evaluacion_Entrega_01.xlsx
+++ b/docs/public/Rubrica_Evaluacion_Entrega_01.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planilla_Notas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seccion_Martes" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz_Rubrica" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escala_Conversion" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,7 +33,7 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="000F172A"/>
-      <sz val="14"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -78,18 +78,12 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <sz val="9"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <color rgb="00334155"/>
       <sz val="9.5"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="000F172A"/>
-      <sz val="13"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -107,11 +101,6 @@
       <b val="1"/>
       <color rgb="000F172A"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <sz val="9.5"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -202,7 +191,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -225,7 +214,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -243,19 +232,16 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -264,19 +250,16 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="15" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="16" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -644,11 +627,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -658,13 +641,13 @@
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="38" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>EVALUACIÓN ENTREGA N°1: ILUMINACIÓN 3-POINT Y SHADER PARAMÉTRICO PBR</t>
+          <t>EVALUACIÓN ENTREGA N°1: ILUMINACIÓN 3-POINT Y SHADER PBR — SECCIÓN MARTES</t>
         </is>
       </c>
     </row>
@@ -682,7 +665,7 @@
         </is>
       </c>
       <c r="C4" s="4">
-        <f>IFERROR(ROUND(AVERAGE(J6:J35), 1), "-")</f>
+        <f>IFERROR(ROUND(AVERAGE(J6:J18), 1), "-")</f>
         <v/>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -691,7 +674,7 @@
         </is>
       </c>
       <c r="E4" s="4">
-        <f>IFERROR(TEXT(COUNTIF(K6:K35, "APROBADO")/MAX(1, COUNTA(B6:B35)), "0.0%"), "0%")</f>
+        <f>IFERROR(TEXT(COUNTIF(K6:K18, "APROBADO")/MAX(1, COUNTA(B6:B18)), "0.0%"), "0%")</f>
         <v/>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -700,7 +683,7 @@
         </is>
       </c>
       <c r="G4" s="4">
-        <f>COUNTIF(K6:K35, "APROBADO") &amp; " / " &amp; COUNTIF(K6:K35, "REPROBADO")</f>
+        <f>COUNTIF(K6:K18, "APROBADO") &amp; " / " &amp; COUNTIF(K6:K18, "REPROBADO")</f>
         <v/>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -709,7 +692,7 @@
         </is>
       </c>
       <c r="I4" s="4">
-        <f>IFERROR(MAX(I6:I35) &amp; " / " &amp; MIN(I6:I35), "-")</f>
+        <f>IFERROR(MAX(I6:I18) &amp; " / " &amp; MIN(I6:I18), "-")</f>
         <v/>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -718,7 +701,7 @@
         </is>
       </c>
       <c r="K4" s="4">
-        <f>IFERROR(MAX(J6:J35) &amp; " / " &amp; MIN(J6:J35), "-")</f>
+        <f>IFERROR(MAX(J6:J18) &amp; " / " &amp; MIN(J6:J18), "-")</f>
         <v/>
       </c>
     </row>
@@ -730,7 +713,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Estudiante (Nombre Completo)</t>
+          <t>Estudiante (Sección Martes)</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -788,37 +771,25 @@
       </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
-          <t>Observaciones y Retroalimentación Docente</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
+          <t>Observaciones y Retroalimentación</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
       <c r="A6" s="7" t="n">
         <v>1</v>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Estudiante Ejemplo 1 (Aprobado)</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="D6" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="E6" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F6" s="9" t="n">
-        <v>14</v>
-      </c>
-      <c r="G6" s="9" t="n">
-        <v>15</v>
-      </c>
-      <c r="H6" s="9" t="n">
-        <v>9</v>
-      </c>
+          <t>JOSE MIGUEL FARFAN CARRASCO</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="n"/>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="9" t="n"/>
       <c r="I6" s="10">
         <f>IF(COUNTA(C6:H6)&gt;0, SUM(C6:H6), "")</f>
         <v/>
@@ -831,39 +802,23 @@
         <f>IF(J6="","",IF(J6&gt;=4.0,"APROBADO","REPROBADO"))</f>
         <v/>
       </c>
-      <c r="L6" s="13" t="inlineStr">
-        <is>
-          <t>Excelente control del modelado y shader PBR bien instanciado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
+      <c r="L6" s="13" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
       <c r="A7" s="7" t="n">
         <v>2</v>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Estudiante Ejemplo 2 (Para Revisión)</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="D7" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="E7" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="F7" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="G7" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="H7" s="9" t="n">
-        <v>5</v>
-      </c>
+          <t>BENJAMIN FERNANDO FIGUEROA GONZALEZ</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="9" t="n"/>
       <c r="I7" s="10">
         <f>IF(COUNTA(C7:H7)&gt;0, SUM(C7:H7), "")</f>
         <v/>
@@ -876,17 +831,17 @@
         <f>IF(J7="","",IF(J7&gt;=4.0,"APROBADO","REPROBADO"))</f>
         <v/>
       </c>
-      <c r="L7" s="13" t="inlineStr">
-        <is>
-          <t>Fill light compite con la Key. Faltan parámetros expuestos en la instancia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
+      <c r="L7" s="13" t="n"/>
+    </row>
+    <row r="8" ht="22" customHeight="1">
       <c r="A8" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="8" t="n"/>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>MATIAS IGNACIO GODOY TIRADO</t>
+        </is>
+      </c>
       <c r="C8" s="9" t="n"/>
       <c r="D8" s="9" t="n"/>
       <c r="E8" s="9" t="n"/>
@@ -907,11 +862,15 @@
       </c>
       <c r="L8" s="13" t="n"/>
     </row>
-    <row r="9" ht="20" customHeight="1">
+    <row r="9" ht="22" customHeight="1">
       <c r="A9" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="8" t="n"/>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>HENRY ALEXANDER HERNANDEZ PEREZ</t>
+        </is>
+      </c>
       <c r="C9" s="9" t="n"/>
       <c r="D9" s="9" t="n"/>
       <c r="E9" s="9" t="n"/>
@@ -932,11 +891,15 @@
       </c>
       <c r="L9" s="13" t="n"/>
     </row>
-    <row r="10" ht="20" customHeight="1">
+    <row r="10" ht="22" customHeight="1">
       <c r="A10" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="8" t="n"/>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>GAEL ALBERTO IBARRA MONTECINOS</t>
+        </is>
+      </c>
       <c r="C10" s="9" t="n"/>
       <c r="D10" s="9" t="n"/>
       <c r="E10" s="9" t="n"/>
@@ -957,11 +920,15 @@
       </c>
       <c r="L10" s="13" t="n"/>
     </row>
-    <row r="11" ht="20" customHeight="1">
+    <row r="11" ht="22" customHeight="1">
       <c r="A11" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="8" t="n"/>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>LUKA PASCAL LATIFE CUEVAS</t>
+        </is>
+      </c>
       <c r="C11" s="9" t="n"/>
       <c r="D11" s="9" t="n"/>
       <c r="E11" s="9" t="n"/>
@@ -982,11 +949,15 @@
       </c>
       <c r="L11" s="13" t="n"/>
     </row>
-    <row r="12" ht="20" customHeight="1">
+    <row r="12" ht="22" customHeight="1">
       <c r="A12" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="8" t="n"/>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>MEI MALDONADO DUARTE</t>
+        </is>
+      </c>
       <c r="C12" s="9" t="n"/>
       <c r="D12" s="9" t="n"/>
       <c r="E12" s="9" t="n"/>
@@ -1007,11 +978,15 @@
       </c>
       <c r="L12" s="13" t="n"/>
     </row>
-    <row r="13" ht="20" customHeight="1">
+    <row r="13" ht="22" customHeight="1">
       <c r="A13" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="8" t="n"/>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>ELIZABETH FABIOLA MEDRANO MORAN</t>
+        </is>
+      </c>
       <c r="C13" s="9" t="n"/>
       <c r="D13" s="9" t="n"/>
       <c r="E13" s="9" t="n"/>
@@ -1032,11 +1007,15 @@
       </c>
       <c r="L13" s="13" t="n"/>
     </row>
-    <row r="14" ht="20" customHeight="1">
+    <row r="14" ht="22" customHeight="1">
       <c r="A14" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="8" t="n"/>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>FREDDY DANILO MONTANARES ROSALES</t>
+        </is>
+      </c>
       <c r="C14" s="9" t="n"/>
       <c r="D14" s="9" t="n"/>
       <c r="E14" s="9" t="n"/>
@@ -1057,11 +1036,15 @@
       </c>
       <c r="L14" s="13" t="n"/>
     </row>
-    <row r="15" ht="20" customHeight="1">
+    <row r="15" ht="22" customHeight="1">
       <c r="A15" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="8" t="n"/>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>JOSE FRANCISCO NAVARRETE BARRIOS</t>
+        </is>
+      </c>
       <c r="C15" s="9" t="n"/>
       <c r="D15" s="9" t="n"/>
       <c r="E15" s="9" t="n"/>
@@ -1082,11 +1065,15 @@
       </c>
       <c r="L15" s="13" t="n"/>
     </row>
-    <row r="16" ht="20" customHeight="1">
+    <row r="16" ht="22" customHeight="1">
       <c r="A16" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="B16" s="8" t="n"/>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>NATANIEL ASTRO REYES FLORES</t>
+        </is>
+      </c>
       <c r="C16" s="9" t="n"/>
       <c r="D16" s="9" t="n"/>
       <c r="E16" s="9" t="n"/>
@@ -1107,11 +1094,15 @@
       </c>
       <c r="L16" s="13" t="n"/>
     </row>
-    <row r="17" ht="20" customHeight="1">
+    <row r="17" ht="22" customHeight="1">
       <c r="A17" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="B17" s="8" t="n"/>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>DANIEL ELIAS ROJAS LOPEZ</t>
+        </is>
+      </c>
       <c r="C17" s="9" t="n"/>
       <c r="D17" s="9" t="n"/>
       <c r="E17" s="9" t="n"/>
@@ -1132,11 +1123,15 @@
       </c>
       <c r="L17" s="13" t="n"/>
     </row>
-    <row r="18" ht="20" customHeight="1">
+    <row r="18" ht="22" customHeight="1">
       <c r="A18" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="B18" s="8" t="n"/>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>CRISTOBAL NICOLAS VALENZUELA PRESSAC</t>
+        </is>
+      </c>
       <c r="C18" s="9" t="n"/>
       <c r="D18" s="9" t="n"/>
       <c r="E18" s="9" t="n"/>
@@ -1156,431 +1151,6 @@
         <v/>
       </c>
       <c r="L18" s="13" t="n"/>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="7" t="n">
-        <v>14</v>
-      </c>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="9" t="n"/>
-      <c r="E19" s="9" t="n"/>
-      <c r="F19" s="9" t="n"/>
-      <c r="G19" s="9" t="n"/>
-      <c r="H19" s="9" t="n"/>
-      <c r="I19" s="10">
-        <f>IF(COUNTA(C19:H19)&gt;0, SUM(C19:H19), "")</f>
-        <v/>
-      </c>
-      <c r="J19" s="11">
-        <f>IF(I19="","",ROUND(IF(I19&lt;36, 1 + 3*(I19/36), 4 + 3*((I19-36)/24)), 1))</f>
-        <v/>
-      </c>
-      <c r="K19" s="12">
-        <f>IF(J19="","",IF(J19&gt;=4.0,"APROBADO","REPROBADO"))</f>
-        <v/>
-      </c>
-      <c r="L19" s="13" t="n"/>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="B20" s="8" t="n"/>
-      <c r="C20" s="9" t="n"/>
-      <c r="D20" s="9" t="n"/>
-      <c r="E20" s="9" t="n"/>
-      <c r="F20" s="9" t="n"/>
-      <c r="G20" s="9" t="n"/>
-      <c r="H20" s="9" t="n"/>
-      <c r="I20" s="10">
-        <f>IF(COUNTA(C20:H20)&gt;0, SUM(C20:H20), "")</f>
-        <v/>
-      </c>
-      <c r="J20" s="11">
-        <f>IF(I20="","",ROUND(IF(I20&lt;36, 1 + 3*(I20/36), 4 + 3*((I20-36)/24)), 1))</f>
-        <v/>
-      </c>
-      <c r="K20" s="12">
-        <f>IF(J20="","",IF(J20&gt;=4.0,"APROBADO","REPROBADO"))</f>
-        <v/>
-      </c>
-      <c r="L20" s="13" t="n"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="7" t="n">
-        <v>16</v>
-      </c>
-      <c r="B21" s="8" t="n"/>
-      <c r="C21" s="9" t="n"/>
-      <c r="D21" s="9" t="n"/>
-      <c r="E21" s="9" t="n"/>
-      <c r="F21" s="9" t="n"/>
-      <c r="G21" s="9" t="n"/>
-      <c r="H21" s="9" t="n"/>
-      <c r="I21" s="10">
-        <f>IF(COUNTA(C21:H21)&gt;0, SUM(C21:H21), "")</f>
-        <v/>
-      </c>
-      <c r="J21" s="11">
-        <f>IF(I21="","",ROUND(IF(I21&lt;36, 1 + 3*(I21/36), 4 + 3*((I21-36)/24)), 1))</f>
-        <v/>
-      </c>
-      <c r="K21" s="12">
-        <f>IF(J21="","",IF(J21&gt;=4.0,"APROBADO","REPROBADO"))</f>
-        <v/>
-      </c>
-      <c r="L21" s="13" t="n"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="7" t="n">
-        <v>17</v>
-      </c>
-      <c r="B22" s="8" t="n"/>
-      <c r="C22" s="9" t="n"/>
-      <c r="D22" s="9" t="n"/>
-      <c r="E22" s="9" t="n"/>
-      <c r="F22" s="9" t="n"/>
-      <c r="G22" s="9" t="n"/>
-      <c r="H22" s="9" t="n"/>
-      <c r="I22" s="10">
-        <f>IF(COUNTA(C22:H22)&gt;0, SUM(C22:H22), "")</f>
-        <v/>
-      </c>
-      <c r="J22" s="11">
-        <f>IF(I22="","",ROUND(IF(I22&lt;36, 1 + 3*(I22/36), 4 + 3*((I22-36)/24)), 1))</f>
-        <v/>
-      </c>
-      <c r="K22" s="12">
-        <f>IF(J22="","",IF(J22&gt;=4.0,"APROBADO","REPROBADO"))</f>
-        <v/>
-      </c>
-      <c r="L22" s="13" t="n"/>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="7" t="n">
-        <v>18</v>
-      </c>
-      <c r="B23" s="8" t="n"/>
-      <c r="C23" s="9" t="n"/>
-      <c r="D23" s="9" t="n"/>
-      <c r="E23" s="9" t="n"/>
-      <c r="F23" s="9" t="n"/>
-      <c r="G23" s="9" t="n"/>
-      <c r="H23" s="9" t="n"/>
-      <c r="I23" s="10">
-        <f>IF(COUNTA(C23:H23)&gt;0, SUM(C23:H23), "")</f>
-        <v/>
-      </c>
-      <c r="J23" s="11">
-        <f>IF(I23="","",ROUND(IF(I23&lt;36, 1 + 3*(I23/36), 4 + 3*((I23-36)/24)), 1))</f>
-        <v/>
-      </c>
-      <c r="K23" s="12">
-        <f>IF(J23="","",IF(J23&gt;=4.0,"APROBADO","REPROBADO"))</f>
-        <v/>
-      </c>
-      <c r="L23" s="13" t="n"/>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="7" t="n">
-        <v>19</v>
-      </c>
-      <c r="B24" s="8" t="n"/>
-      <c r="C24" s="9" t="n"/>
-      <c r="D24" s="9" t="n"/>
-      <c r="E24" s="9" t="n"/>
-      <c r="F24" s="9" t="n"/>
-      <c r="G24" s="9" t="n"/>
-      <c r="H24" s="9" t="n"/>
-      <c r="I24" s="10">
-        <f>IF(COUNTA(C24:H24)&gt;0, SUM(C24:H24), "")</f>
-        <v/>
-      </c>
-      <c r="J24" s="11">
-        <f>IF(I24="","",ROUND(IF(I24&lt;36, 1 + 3*(I24/36), 4 + 3*((I24-36)/24)), 1))</f>
-        <v/>
-      </c>
-      <c r="K24" s="12">
-        <f>IF(J24="","",IF(J24&gt;=4.0,"APROBADO","REPROBADO"))</f>
-        <v/>
-      </c>
-      <c r="L24" s="13" t="n"/>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="B25" s="8" t="n"/>
-      <c r="C25" s="9" t="n"/>
-      <c r="D25" s="9" t="n"/>
-      <c r="E25" s="9" t="n"/>
-      <c r="F25" s="9" t="n"/>
-      <c r="G25" s="9" t="n"/>
-      <c r="H25" s="9" t="n"/>
-      <c r="I25" s="10">
-        <f>IF(COUNTA(C25:H25)&gt;0, SUM(C25:H25), "")</f>
-        <v/>
-      </c>
-      <c r="J25" s="11">
-        <f>IF(I25="","",ROUND(IF(I25&lt;36, 1 + 3*(I25/36), 4 + 3*((I25-36)/24)), 1))</f>
-        <v/>
-      </c>
-      <c r="K25" s="12">
-        <f>IF(J25="","",IF(J25&gt;=4.0,"APROBADO","REPROBADO"))</f>
-        <v/>
-      </c>
-      <c r="L25" s="13" t="n"/>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="7" t="n">
-        <v>21</v>
-      </c>
-      <c r="B26" s="8" t="n"/>
-      <c r="C26" s="9" t="n"/>
-      <c r="D26" s="9" t="n"/>
-      <c r="E26" s="9" t="n"/>
-      <c r="F26" s="9" t="n"/>
-      <c r="G26" s="9" t="n"/>
-      <c r="H26" s="9" t="n"/>
-      <c r="I26" s="10">
-        <f>IF(COUNTA(C26:H26)&gt;0, SUM(C26:H26), "")</f>
-        <v/>
-      </c>
-      <c r="J26" s="11">
-        <f>IF(I26="","",ROUND(IF(I26&lt;36, 1 + 3*(I26/36), 4 + 3*((I26-36)/24)), 1))</f>
-        <v/>
-      </c>
-      <c r="K26" s="12">
-        <f>IF(J26="","",IF(J26&gt;=4.0,"APROBADO","REPROBADO"))</f>
-        <v/>
-      </c>
-      <c r="L26" s="13" t="n"/>
-    </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="B27" s="8" t="n"/>
-      <c r="C27" s="9" t="n"/>
-      <c r="D27" s="9" t="n"/>
-      <c r="E27" s="9" t="n"/>
-      <c r="F27" s="9" t="n"/>
-      <c r="G27" s="9" t="n"/>
-      <c r="H27" s="9" t="n"/>
-      <c r="I27" s="10">
-        <f>IF(COUNTA(C27:H27)&gt;0, SUM(C27:H27), "")</f>
-        <v/>
-      </c>
-      <c r="J27" s="11">
-        <f>IF(I27="","",ROUND(IF(I27&lt;36, 1 + 3*(I27/36), 4 + 3*((I27-36)/24)), 1))</f>
-        <v/>
-      </c>
-      <c r="K27" s="12">
-        <f>IF(J27="","",IF(J27&gt;=4.0,"APROBADO","REPROBADO"))</f>
-        <v/>
-      </c>
-      <c r="L27" s="13" t="n"/>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="7" t="n">
-        <v>23</v>
-      </c>
-      <c r="B28" s="8" t="n"/>
-      <c r="C28" s="9" t="n"/>
-      <c r="D28" s="9" t="n"/>
-      <c r="E28" s="9" t="n"/>
-      <c r="F28" s="9" t="n"/>
-      <c r="G28" s="9" t="n"/>
-      <c r="H28" s="9" t="n"/>
-      <c r="I28" s="10">
-        <f>IF(COUNTA(C28:H28)&gt;0, SUM(C28:H28), "")</f>
-        <v/>
-      </c>
-      <c r="J28" s="11">
-        <f>IF(I28="","",ROUND(IF(I28&lt;36, 1 + 3*(I28/36), 4 + 3*((I28-36)/24)), 1))</f>
-        <v/>
-      </c>
-      <c r="K28" s="12">
-        <f>IF(J28="","",IF(J28&gt;=4.0,"APROBADO","REPROBADO"))</f>
-        <v/>
-      </c>
-      <c r="L28" s="13" t="n"/>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="7" t="n">
-        <v>24</v>
-      </c>
-      <c r="B29" s="8" t="n"/>
-      <c r="C29" s="9" t="n"/>
-      <c r="D29" s="9" t="n"/>
-      <c r="E29" s="9" t="n"/>
-      <c r="F29" s="9" t="n"/>
-      <c r="G29" s="9" t="n"/>
-      <c r="H29" s="9" t="n"/>
-      <c r="I29" s="10">
-        <f>IF(COUNTA(C29:H29)&gt;0, SUM(C29:H29), "")</f>
-        <v/>
-      </c>
-      <c r="J29" s="11">
-        <f>IF(I29="","",ROUND(IF(I29&lt;36, 1 + 3*(I29/36), 4 + 3*((I29-36)/24)), 1))</f>
-        <v/>
-      </c>
-      <c r="K29" s="12">
-        <f>IF(J29="","",IF(J29&gt;=4.0,"APROBADO","REPROBADO"))</f>
-        <v/>
-      </c>
-      <c r="L29" s="13" t="n"/>
-    </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="7" t="n">
-        <v>25</v>
-      </c>
-      <c r="B30" s="8" t="n"/>
-      <c r="C30" s="9" t="n"/>
-      <c r="D30" s="9" t="n"/>
-      <c r="E30" s="9" t="n"/>
-      <c r="F30" s="9" t="n"/>
-      <c r="G30" s="9" t="n"/>
-      <c r="H30" s="9" t="n"/>
-      <c r="I30" s="10">
-        <f>IF(COUNTA(C30:H30)&gt;0, SUM(C30:H30), "")</f>
-        <v/>
-      </c>
-      <c r="J30" s="11">
-        <f>IF(I30="","",ROUND(IF(I30&lt;36, 1 + 3*(I30/36), 4 + 3*((I30-36)/24)), 1))</f>
-        <v/>
-      </c>
-      <c r="K30" s="12">
-        <f>IF(J30="","",IF(J30&gt;=4.0,"APROBADO","REPROBADO"))</f>
-        <v/>
-      </c>
-      <c r="L30" s="13" t="n"/>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="7" t="n">
-        <v>26</v>
-      </c>
-      <c r="B31" s="8" t="n"/>
-      <c r="C31" s="9" t="n"/>
-      <c r="D31" s="9" t="n"/>
-      <c r="E31" s="9" t="n"/>
-      <c r="F31" s="9" t="n"/>
-      <c r="G31" s="9" t="n"/>
-      <c r="H31" s="9" t="n"/>
-      <c r="I31" s="10">
-        <f>IF(COUNTA(C31:H31)&gt;0, SUM(C31:H31), "")</f>
-        <v/>
-      </c>
-      <c r="J31" s="11">
-        <f>IF(I31="","",ROUND(IF(I31&lt;36, 1 + 3*(I31/36), 4 + 3*((I31-36)/24)), 1))</f>
-        <v/>
-      </c>
-      <c r="K31" s="12">
-        <f>IF(J31="","",IF(J31&gt;=4.0,"APROBADO","REPROBADO"))</f>
-        <v/>
-      </c>
-      <c r="L31" s="13" t="n"/>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="7" t="n">
-        <v>27</v>
-      </c>
-      <c r="B32" s="8" t="n"/>
-      <c r="C32" s="9" t="n"/>
-      <c r="D32" s="9" t="n"/>
-      <c r="E32" s="9" t="n"/>
-      <c r="F32" s="9" t="n"/>
-      <c r="G32" s="9" t="n"/>
-      <c r="H32" s="9" t="n"/>
-      <c r="I32" s="10">
-        <f>IF(COUNTA(C32:H32)&gt;0, SUM(C32:H32), "")</f>
-        <v/>
-      </c>
-      <c r="J32" s="11">
-        <f>IF(I32="","",ROUND(IF(I32&lt;36, 1 + 3*(I32/36), 4 + 3*((I32-36)/24)), 1))</f>
-        <v/>
-      </c>
-      <c r="K32" s="12">
-        <f>IF(J32="","",IF(J32&gt;=4.0,"APROBADO","REPROBADO"))</f>
-        <v/>
-      </c>
-      <c r="L32" s="13" t="n"/>
-    </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="7" t="n">
-        <v>28</v>
-      </c>
-      <c r="B33" s="8" t="n"/>
-      <c r="C33" s="9" t="n"/>
-      <c r="D33" s="9" t="n"/>
-      <c r="E33" s="9" t="n"/>
-      <c r="F33" s="9" t="n"/>
-      <c r="G33" s="9" t="n"/>
-      <c r="H33" s="9" t="n"/>
-      <c r="I33" s="10">
-        <f>IF(COUNTA(C33:H33)&gt;0, SUM(C33:H33), "")</f>
-        <v/>
-      </c>
-      <c r="J33" s="11">
-        <f>IF(I33="","",ROUND(IF(I33&lt;36, 1 + 3*(I33/36), 4 + 3*((I33-36)/24)), 1))</f>
-        <v/>
-      </c>
-      <c r="K33" s="12">
-        <f>IF(J33="","",IF(J33&gt;=4.0,"APROBADO","REPROBADO"))</f>
-        <v/>
-      </c>
-      <c r="L33" s="13" t="n"/>
-    </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="7" t="n">
-        <v>29</v>
-      </c>
-      <c r="B34" s="8" t="n"/>
-      <c r="C34" s="9" t="n"/>
-      <c r="D34" s="9" t="n"/>
-      <c r="E34" s="9" t="n"/>
-      <c r="F34" s="9" t="n"/>
-      <c r="G34" s="9" t="n"/>
-      <c r="H34" s="9" t="n"/>
-      <c r="I34" s="10">
-        <f>IF(COUNTA(C34:H34)&gt;0, SUM(C34:H34), "")</f>
-        <v/>
-      </c>
-      <c r="J34" s="11">
-        <f>IF(I34="","",ROUND(IF(I34&lt;36, 1 + 3*(I34/36), 4 + 3*((I34-36)/24)), 1))</f>
-        <v/>
-      </c>
-      <c r="K34" s="12">
-        <f>IF(J34="","",IF(J34&gt;=4.0,"APROBADO","REPROBADO"))</f>
-        <v/>
-      </c>
-      <c r="L34" s="13" t="n"/>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="B35" s="8" t="n"/>
-      <c r="C35" s="9" t="n"/>
-      <c r="D35" s="9" t="n"/>
-      <c r="E35" s="9" t="n"/>
-      <c r="F35" s="9" t="n"/>
-      <c r="G35" s="9" t="n"/>
-      <c r="H35" s="9" t="n"/>
-      <c r="I35" s="10">
-        <f>IF(COUNTA(C35:H35)&gt;0, SUM(C35:H35), "")</f>
-        <v/>
-      </c>
-      <c r="J35" s="11">
-        <f>IF(I35="","",ROUND(IF(I35&lt;36, 1 + 3*(I35/36), 4 + 3*((I35-36)/24)), 1))</f>
-        <v/>
-      </c>
-      <c r="K35" s="12">
-        <f>IF(J35="","",IF(J35&gt;=4.0,"APROBADO","REPROBADO"))</f>
-        <v/>
-      </c>
-      <c r="L35" s="13" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1609,7 +1179,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>MATRIZ DESCRIPTIVA DE EVALUACIÓN (TOTAL: 60 PUNTOS)</t>
         </is>
@@ -1648,192 +1218,192 @@
       </c>
     </row>
     <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>1. Key Light (Luz Principal)</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Posicionada a ~45° lateral y cenital. Define claramente el modelado volumétrico, contraste y dirección de sombras sin sobreexponer.</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>Posicionada adecuadamente pero con leve descalibración de intensidad (zonas ligeramente quemadas o sombra poco definida).</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>Ubicación incorrecta o intensidad muy baja/alta, afectando la lectura del volumen del objeto.</t>
         </is>
       </c>
-      <c r="E4" s="16" t="inlineStr">
+      <c r="E4" s="15" t="inlineStr">
         <is>
           <t>Luz ausente, mal orientada o que no cumple el rol de emisor dominante.</t>
         </is>
       </c>
-      <c r="F4" s="17" t="inlineStr">
+      <c r="F4" s="16" t="inlineStr">
         <is>
           <t>7 pts</t>
         </is>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>2. Fill Light (Luz de Relleno)</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>Ubicada en el flanco opuesto. Intensidad calibrada (25-40% de Key). Suaviza sombras duras rescatando información sin generar sombras cruzadas.</t>
         </is>
       </c>
-      <c r="C5" s="16" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>Ubicada correctamente pero su intensidad compite con Key (&gt;50%) o es demasiado tenue (&lt;15%).</t>
         </is>
       </c>
-      <c r="D5" s="16" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>Genera sombras cruzadas notorias o no logra levantar la penumbra del lado oscuro.</t>
         </is>
       </c>
-      <c r="E5" s="16" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
         <is>
           <t>Ausente o colocada en posición errónea que anula el contraste del esquema.</t>
         </is>
       </c>
-      <c r="F5" s="17" t="inlineStr">
+      <c r="F5" s="16" t="inlineStr">
         <is>
           <t>7 pts</t>
         </is>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>3. Rim Light (Contraluz)</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Ubicada detrás del sujeto. Dibuja un filete brillante limpio y continuo en bordes y hombros, separando perfectamente del fondo oscuro.</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>Presente y bien ubicada, pero con intensidad algo excesiva (quema el contorno) o muy tenue.</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>Posición deficiente; solo ilumina una fracción menor del borde sin lograr despegar el modelo.</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>Ausente o no genera contraste de silueta respecto al fondo.</t>
         </is>
       </c>
-      <c r="F6" s="17" t="inlineStr">
+      <c r="F6" s="16" t="inlineStr">
         <is>
           <t>6 pts</t>
         </is>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>4. Material PBR y Texturizado</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>Mapas de textura (BaseColor, Normal, ORM) asignados correctamente. Respuesta física coherente y verosímil según el material.</t>
         </is>
       </c>
-      <c r="C7" s="16" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>Texturas bien asignadas pero con leves desajustes en el balance de rugosidad o fuerza de normales.</t>
         </is>
       </c>
-      <c r="D7" s="16" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>Errores en la asignación de canales (ej. Normal Map invertido o rugosidad no calibrada).</t>
         </is>
       </c>
-      <c r="E7" s="16" t="inlineStr">
+      <c r="E7" s="15" t="inlineStr">
         <is>
           <t>Material plano sin mapas PBR o texturas con sombras pintadas a mano que rompen el PBR.</t>
         </is>
       </c>
-      <c r="F7" s="17" t="inlineStr">
+      <c r="F7" s="16" t="inlineStr">
         <is>
           <t>15 pts</t>
         </is>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>5. Arquitectura del Shader e Instancias</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>Construcción correcta de Master Material (M_) y derivación a Instancia (MI_). Presenta 3 o más parámetros expuestos y funcionales en tiempo real.</t>
         </is>
       </c>
-      <c r="C8" s="16" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr">
         <is>
           <t>Presenta Master e Instancia, pero solo 2 parámetros funcionan correctamente o su nomenclatura es genérica.</t>
         </is>
       </c>
-      <c r="D8" s="16" t="inlineStr">
+      <c r="D8" s="15" t="inlineStr">
         <is>
           <t>Material con solo 1 parámetro expuesto o no utiliza el flujo de instancias (modifica el shader base).</t>
         </is>
       </c>
-      <c r="E8" s="16" t="inlineStr">
+      <c r="E8" s="15" t="inlineStr">
         <is>
           <t>No utiliza instancias de material ni expone parámetros escalares/vectoriales.</t>
         </is>
       </c>
-      <c r="F8" s="17" t="inlineStr">
+      <c r="F8" s="16" t="inlineStr">
         <is>
           <t>15 pts</t>
         </is>
       </c>
     </row>
     <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>6. Nomenclatura, Orden y Presentación</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>Proyecto ordenado con nomenclatura estándar de la industria (M_, MI_, T_, SM_, L_). Outliner limpio. Renders nítidos y bien encuadrados.</t>
         </is>
       </c>
-      <c r="C9" s="16" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>Proyecto comprensible pero con descuidos menores en nomenclatura o carpetas.</t>
         </is>
       </c>
-      <c r="D9" s="16" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>Desorden evidente en el árbol de contenido o nombres por defecto (NewMaterial, PointLight1).</t>
         </is>
       </c>
-      <c r="E9" s="16" t="inlineStr">
+      <c r="E9" s="15" t="inlineStr">
         <is>
           <t>Proyecto desorganizado, archivos rotos o faltan capturas solicitadas.</t>
         </is>
       </c>
-      <c r="F9" s="17" t="inlineStr">
+      <c r="F9" s="16" t="inlineStr">
         <is>
           <t>10 pts</t>
         </is>
@@ -1863,1127 +1433,1127 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="18" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>TABLA DE CONVERSIÓN OFICIAL: PUNTAJE A NOTA CHILENA (1.0 A 7.0 AL 60%)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>Puntaje (pts)</t>
         </is>
       </c>
-      <c r="B3" s="19" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>% Logro</t>
         </is>
       </c>
-      <c r="C3" s="19" t="inlineStr">
+      <c r="C3" s="18" t="inlineStr">
         <is>
           <t>Nota Final</t>
         </is>
       </c>
-      <c r="D3" s="20" t="inlineStr">
+      <c r="D3" s="19" t="inlineStr">
         <is>
           <t>Nivel de Desempeño</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="21" t="n">
+      <c r="A4" s="12" t="n">
         <v>60</v>
       </c>
-      <c r="B4" s="22" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="C4" s="23" t="n">
+      <c r="C4" s="21" t="n">
         <v>7</v>
       </c>
-      <c r="D4" s="24" t="inlineStr">
+      <c r="D4" s="22" t="inlineStr">
         <is>
           <t>Sobresaliente</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="21" t="n">
+      <c r="A5" s="12" t="n">
         <v>59</v>
       </c>
-      <c r="B5" s="22" t="inlineStr">
+      <c r="B5" s="20" t="inlineStr">
         <is>
           <t>98.3%</t>
         </is>
       </c>
-      <c r="C5" s="23" t="n">
+      <c r="C5" s="21" t="n">
         <v>6.9</v>
       </c>
-      <c r="D5" s="24" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>Sobresaliente</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="21" t="n">
+      <c r="A6" s="12" t="n">
         <v>58</v>
       </c>
-      <c r="B6" s="22" t="inlineStr">
+      <c r="B6" s="20" t="inlineStr">
         <is>
           <t>96.7%</t>
         </is>
       </c>
-      <c r="C6" s="23" t="n">
+      <c r="C6" s="21" t="n">
         <v>6.8</v>
       </c>
-      <c r="D6" s="24" t="inlineStr">
+      <c r="D6" s="22" t="inlineStr">
         <is>
           <t>Sobresaliente</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="21" t="n">
+      <c r="A7" s="12" t="n">
         <v>57</v>
       </c>
-      <c r="B7" s="22" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>95.0%</t>
         </is>
       </c>
-      <c r="C7" s="23" t="n">
+      <c r="C7" s="21" t="n">
         <v>6.6</v>
       </c>
-      <c r="D7" s="24" t="inlineStr">
+      <c r="D7" s="22" t="inlineStr">
         <is>
           <t>Sobresaliente</t>
         </is>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="21" t="n">
+      <c r="A8" s="12" t="n">
         <v>56</v>
       </c>
-      <c r="B8" s="22" t="inlineStr">
+      <c r="B8" s="20" t="inlineStr">
         <is>
           <t>93.3%</t>
         </is>
       </c>
-      <c r="C8" s="23" t="n">
+      <c r="C8" s="21" t="n">
         <v>6.5</v>
       </c>
-      <c r="D8" s="24" t="inlineStr">
+      <c r="D8" s="22" t="inlineStr">
         <is>
           <t>Sobresaliente</t>
         </is>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="21" t="n">
+      <c r="A9" s="12" t="n">
         <v>55</v>
       </c>
-      <c r="B9" s="22" t="inlineStr">
+      <c r="B9" s="20" t="inlineStr">
         <is>
           <t>91.7%</t>
         </is>
       </c>
-      <c r="C9" s="23" t="n">
+      <c r="C9" s="21" t="n">
         <v>6.4</v>
       </c>
-      <c r="D9" s="24" t="inlineStr">
+      <c r="D9" s="22" t="inlineStr">
         <is>
           <t>Muy Bueno</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="21" t="n">
+      <c r="A10" s="12" t="n">
         <v>54</v>
       </c>
-      <c r="B10" s="22" t="inlineStr">
+      <c r="B10" s="20" t="inlineStr">
         <is>
           <t>90.0%</t>
         </is>
       </c>
-      <c r="C10" s="23" t="n">
+      <c r="C10" s="21" t="n">
         <v>6.2</v>
       </c>
-      <c r="D10" s="24" t="inlineStr">
+      <c r="D10" s="22" t="inlineStr">
         <is>
           <t>Muy Bueno</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="21" t="n">
+      <c r="A11" s="12" t="n">
         <v>53</v>
       </c>
-      <c r="B11" s="22" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>88.3%</t>
         </is>
       </c>
-      <c r="C11" s="23" t="n">
+      <c r="C11" s="21" t="n">
         <v>6.1</v>
       </c>
-      <c r="D11" s="24" t="inlineStr">
+      <c r="D11" s="22" t="inlineStr">
         <is>
           <t>Muy Bueno</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="21" t="n">
+      <c r="A12" s="12" t="n">
         <v>52</v>
       </c>
-      <c r="B12" s="22" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>86.7%</t>
         </is>
       </c>
-      <c r="C12" s="23" t="n">
+      <c r="C12" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="D12" s="24" t="inlineStr">
+      <c r="D12" s="22" t="inlineStr">
         <is>
           <t>Muy Bueno</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="21" t="n">
+      <c r="A13" s="12" t="n">
         <v>51</v>
       </c>
-      <c r="B13" s="22" t="inlineStr">
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>85.0%</t>
         </is>
       </c>
-      <c r="C13" s="23" t="n">
+      <c r="C13" s="21" t="n">
         <v>5.9</v>
       </c>
-      <c r="D13" s="24" t="inlineStr">
+      <c r="D13" s="22" t="inlineStr">
         <is>
           <t>Muy Bueno</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="21" t="n">
+      <c r="A14" s="12" t="n">
         <v>50</v>
       </c>
-      <c r="B14" s="22" t="inlineStr">
+      <c r="B14" s="20" t="inlineStr">
         <is>
           <t>83.3%</t>
         </is>
       </c>
-      <c r="C14" s="23" t="n">
+      <c r="C14" s="21" t="n">
         <v>5.8</v>
       </c>
-      <c r="D14" s="24" t="inlineStr">
+      <c r="D14" s="22" t="inlineStr">
         <is>
           <t>Muy Bueno</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="21" t="n">
+      <c r="A15" s="12" t="n">
         <v>49</v>
       </c>
-      <c r="B15" s="22" t="inlineStr">
+      <c r="B15" s="20" t="inlineStr">
         <is>
           <t>81.7%</t>
         </is>
       </c>
-      <c r="C15" s="23" t="n">
+      <c r="C15" s="21" t="n">
         <v>5.6</v>
       </c>
-      <c r="D15" s="24" t="inlineStr">
+      <c r="D15" s="22" t="inlineStr">
         <is>
           <t>Bueno</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="21" t="n">
+      <c r="A16" s="12" t="n">
         <v>48</v>
       </c>
-      <c r="B16" s="22" t="inlineStr">
+      <c r="B16" s="20" t="inlineStr">
         <is>
           <t>80.0%</t>
         </is>
       </c>
-      <c r="C16" s="23" t="n">
+      <c r="C16" s="21" t="n">
         <v>5.5</v>
       </c>
-      <c r="D16" s="24" t="inlineStr">
+      <c r="D16" s="22" t="inlineStr">
         <is>
           <t>Bueno</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="21" t="n">
+      <c r="A17" s="12" t="n">
         <v>47</v>
       </c>
-      <c r="B17" s="22" t="inlineStr">
+      <c r="B17" s="20" t="inlineStr">
         <is>
           <t>78.3%</t>
         </is>
       </c>
-      <c r="C17" s="23" t="n">
+      <c r="C17" s="21" t="n">
         <v>5.4</v>
       </c>
-      <c r="D17" s="24" t="inlineStr">
+      <c r="D17" s="22" t="inlineStr">
         <is>
           <t>Bueno</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="21" t="n">
+      <c r="A18" s="12" t="n">
         <v>46</v>
       </c>
-      <c r="B18" s="22" t="inlineStr">
+      <c r="B18" s="20" t="inlineStr">
         <is>
           <t>76.7%</t>
         </is>
       </c>
-      <c r="C18" s="23" t="n">
+      <c r="C18" s="21" t="n">
         <v>5.2</v>
       </c>
-      <c r="D18" s="24" t="inlineStr">
+      <c r="D18" s="22" t="inlineStr">
         <is>
           <t>Bueno</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="21" t="n">
+      <c r="A19" s="12" t="n">
         <v>45</v>
       </c>
-      <c r="B19" s="22" t="inlineStr">
+      <c r="B19" s="20" t="inlineStr">
         <is>
           <t>75.0%</t>
         </is>
       </c>
-      <c r="C19" s="23" t="n">
+      <c r="C19" s="21" t="n">
         <v>5.1</v>
       </c>
-      <c r="D19" s="24" t="inlineStr">
+      <c r="D19" s="22" t="inlineStr">
         <is>
           <t>Bueno</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="21" t="n">
+      <c r="A20" s="12" t="n">
         <v>44</v>
       </c>
-      <c r="B20" s="22" t="inlineStr">
+      <c r="B20" s="20" t="inlineStr">
         <is>
           <t>73.3%</t>
         </is>
       </c>
-      <c r="C20" s="23" t="n">
+      <c r="C20" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="D20" s="24" t="inlineStr">
+      <c r="D20" s="22" t="inlineStr">
         <is>
           <t>Bueno</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="21" t="n">
+      <c r="A21" s="12" t="n">
         <v>43</v>
       </c>
-      <c r="B21" s="22" t="inlineStr">
+      <c r="B21" s="20" t="inlineStr">
         <is>
           <t>71.7%</t>
         </is>
       </c>
-      <c r="C21" s="23" t="n">
+      <c r="C21" s="21" t="n">
         <v>4.9</v>
       </c>
-      <c r="D21" s="24" t="inlineStr">
+      <c r="D21" s="22" t="inlineStr">
         <is>
           <t>Aprobado (Suficiente)</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="21" t="n">
+      <c r="A22" s="12" t="n">
         <v>42</v>
       </c>
-      <c r="B22" s="22" t="inlineStr">
+      <c r="B22" s="20" t="inlineStr">
         <is>
           <t>70.0%</t>
         </is>
       </c>
-      <c r="C22" s="23" t="n">
+      <c r="C22" s="21" t="n">
         <v>4.8</v>
       </c>
-      <c r="D22" s="24" t="inlineStr">
+      <c r="D22" s="22" t="inlineStr">
         <is>
           <t>Aprobado (Suficiente)</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="21" t="n">
+      <c r="A23" s="12" t="n">
         <v>41</v>
       </c>
-      <c r="B23" s="22" t="inlineStr">
+      <c r="B23" s="20" t="inlineStr">
         <is>
           <t>68.3%</t>
         </is>
       </c>
-      <c r="C23" s="23" t="n">
+      <c r="C23" s="21" t="n">
         <v>4.6</v>
       </c>
-      <c r="D23" s="24" t="inlineStr">
+      <c r="D23" s="22" t="inlineStr">
         <is>
           <t>Aprobado (Suficiente)</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="21" t="n">
+      <c r="A24" s="12" t="n">
         <v>40</v>
       </c>
-      <c r="B24" s="22" t="inlineStr">
+      <c r="B24" s="20" t="inlineStr">
         <is>
           <t>66.7%</t>
         </is>
       </c>
-      <c r="C24" s="23" t="n">
+      <c r="C24" s="21" t="n">
         <v>4.5</v>
       </c>
-      <c r="D24" s="24" t="inlineStr">
+      <c r="D24" s="22" t="inlineStr">
         <is>
           <t>Aprobado (Suficiente)</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="21" t="n">
+      <c r="A25" s="12" t="n">
         <v>39</v>
       </c>
-      <c r="B25" s="22" t="inlineStr">
+      <c r="B25" s="20" t="inlineStr">
         <is>
           <t>65.0%</t>
         </is>
       </c>
-      <c r="C25" s="23" t="n">
+      <c r="C25" s="21" t="n">
         <v>4.4</v>
       </c>
-      <c r="D25" s="24" t="inlineStr">
+      <c r="D25" s="22" t="inlineStr">
         <is>
           <t>Aprobado (Suficiente)</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="21" t="n">
+      <c r="A26" s="12" t="n">
         <v>38</v>
       </c>
-      <c r="B26" s="22" t="inlineStr">
+      <c r="B26" s="20" t="inlineStr">
         <is>
           <t>63.3%</t>
         </is>
       </c>
-      <c r="C26" s="23" t="n">
+      <c r="C26" s="21" t="n">
         <v>4.2</v>
       </c>
-      <c r="D26" s="24" t="inlineStr">
+      <c r="D26" s="22" t="inlineStr">
         <is>
           <t>Aprobado (Suficiente)</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="21" t="n">
+      <c r="A27" s="12" t="n">
         <v>37</v>
       </c>
-      <c r="B27" s="22" t="inlineStr">
+      <c r="B27" s="20" t="inlineStr">
         <is>
           <t>61.7%</t>
         </is>
       </c>
-      <c r="C27" s="23" t="n">
+      <c r="C27" s="21" t="n">
         <v>4.1</v>
       </c>
-      <c r="D27" s="24" t="inlineStr">
+      <c r="D27" s="22" t="inlineStr">
         <is>
           <t>Aprobado (Suficiente)</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="21" t="n">
+      <c r="A28" s="12" t="n">
         <v>36</v>
       </c>
-      <c r="B28" s="22" t="inlineStr">
+      <c r="B28" s="20" t="inlineStr">
         <is>
           <t>60.0%</t>
         </is>
       </c>
-      <c r="C28" s="23" t="n">
+      <c r="C28" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="D28" s="24" t="inlineStr">
+      <c r="D28" s="22" t="inlineStr">
         <is>
           <t>Aprobado (Suficiente)</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="21" t="n">
+      <c r="A29" s="12" t="n">
         <v>35</v>
       </c>
-      <c r="B29" s="22" t="inlineStr">
+      <c r="B29" s="20" t="inlineStr">
         <is>
           <t>58.3%</t>
         </is>
       </c>
-      <c r="C29" s="25" t="n">
+      <c r="C29" s="23" t="n">
         <v>3.9</v>
       </c>
-      <c r="D29" s="24" t="inlineStr">
+      <c r="D29" s="22" t="inlineStr">
         <is>
           <t>Reprobado (Insuficiente)</t>
         </is>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="21" t="n">
+      <c r="A30" s="12" t="n">
         <v>34</v>
       </c>
-      <c r="B30" s="22" t="inlineStr">
+      <c r="B30" s="20" t="inlineStr">
         <is>
           <t>56.7%</t>
         </is>
       </c>
-      <c r="C30" s="25" t="n">
+      <c r="C30" s="23" t="n">
         <v>3.8</v>
       </c>
-      <c r="D30" s="24" t="inlineStr">
+      <c r="D30" s="22" t="inlineStr">
         <is>
           <t>Reprobado (Insuficiente)</t>
         </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="21" t="n">
+      <c r="A31" s="12" t="n">
         <v>33</v>
       </c>
-      <c r="B31" s="22" t="inlineStr">
+      <c r="B31" s="20" t="inlineStr">
         <is>
           <t>55.0%</t>
         </is>
       </c>
-      <c r="C31" s="25" t="n">
+      <c r="C31" s="23" t="n">
         <v>3.8</v>
       </c>
-      <c r="D31" s="24" t="inlineStr">
+      <c r="D31" s="22" t="inlineStr">
         <is>
           <t>Reprobado (Insuficiente)</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="21" t="n">
+      <c r="A32" s="12" t="n">
         <v>32</v>
       </c>
-      <c r="B32" s="22" t="inlineStr">
+      <c r="B32" s="20" t="inlineStr">
         <is>
           <t>53.3%</t>
         </is>
       </c>
-      <c r="C32" s="25" t="n">
+      <c r="C32" s="23" t="n">
         <v>3.7</v>
       </c>
-      <c r="D32" s="24" t="inlineStr">
+      <c r="D32" s="22" t="inlineStr">
         <is>
           <t>Reprobado (Insuficiente)</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="21" t="n">
+      <c r="A33" s="12" t="n">
         <v>31</v>
       </c>
-      <c r="B33" s="22" t="inlineStr">
+      <c r="B33" s="20" t="inlineStr">
         <is>
           <t>51.7%</t>
         </is>
       </c>
-      <c r="C33" s="25" t="n">
+      <c r="C33" s="23" t="n">
         <v>3.6</v>
       </c>
-      <c r="D33" s="24" t="inlineStr">
+      <c r="D33" s="22" t="inlineStr">
         <is>
           <t>Reprobado (Insuficiente)</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="21" t="n">
+      <c r="A34" s="12" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="22" t="inlineStr">
+      <c r="B34" s="20" t="inlineStr">
         <is>
           <t>50.0%</t>
         </is>
       </c>
-      <c r="C34" s="25" t="n">
+      <c r="C34" s="23" t="n">
         <v>3.5</v>
       </c>
-      <c r="D34" s="24" t="inlineStr">
+      <c r="D34" s="22" t="inlineStr">
         <is>
           <t>Reprobado (Insuficiente)</t>
         </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="21" t="n">
+      <c r="A35" s="12" t="n">
         <v>29</v>
       </c>
-      <c r="B35" s="22" t="inlineStr">
+      <c r="B35" s="20" t="inlineStr">
         <is>
           <t>48.3%</t>
         </is>
       </c>
-      <c r="C35" s="25" t="n">
+      <c r="C35" s="23" t="n">
         <v>3.4</v>
       </c>
-      <c r="D35" s="24" t="inlineStr">
+      <c r="D35" s="22" t="inlineStr">
         <is>
           <t>Reprobado (Insuficiente)</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="21" t="n">
+      <c r="A36" s="12" t="n">
         <v>28</v>
       </c>
-      <c r="B36" s="22" t="inlineStr">
+      <c r="B36" s="20" t="inlineStr">
         <is>
           <t>46.7%</t>
         </is>
       </c>
-      <c r="C36" s="25" t="n">
+      <c r="C36" s="23" t="n">
         <v>3.3</v>
       </c>
-      <c r="D36" s="24" t="inlineStr">
+      <c r="D36" s="22" t="inlineStr">
         <is>
           <t>Reprobado (Insuficiente)</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="21" t="n">
+      <c r="A37" s="12" t="n">
         <v>27</v>
       </c>
-      <c r="B37" s="22" t="inlineStr">
+      <c r="B37" s="20" t="inlineStr">
         <is>
           <t>45.0%</t>
         </is>
       </c>
-      <c r="C37" s="25" t="n">
+      <c r="C37" s="23" t="n">
         <v>3.2</v>
       </c>
-      <c r="D37" s="24" t="inlineStr">
+      <c r="D37" s="22" t="inlineStr">
         <is>
           <t>Reprobado (Insuficiente)</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="21" t="n">
+      <c r="A38" s="12" t="n">
         <v>26</v>
       </c>
-      <c r="B38" s="22" t="inlineStr">
+      <c r="B38" s="20" t="inlineStr">
         <is>
           <t>43.3%</t>
         </is>
       </c>
-      <c r="C38" s="25" t="n">
+      <c r="C38" s="23" t="n">
         <v>3.2</v>
       </c>
-      <c r="D38" s="24" t="inlineStr">
+      <c r="D38" s="22" t="inlineStr">
         <is>
           <t>Reprobado (Insuficiente)</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="21" t="n">
+      <c r="A39" s="12" t="n">
         <v>25</v>
       </c>
-      <c r="B39" s="22" t="inlineStr">
+      <c r="B39" s="20" t="inlineStr">
         <is>
           <t>41.7%</t>
         </is>
       </c>
-      <c r="C39" s="25" t="n">
+      <c r="C39" s="23" t="n">
         <v>3.1</v>
       </c>
-      <c r="D39" s="24" t="inlineStr">
+      <c r="D39" s="22" t="inlineStr">
         <is>
           <t>Reprobado (Insuficiente)</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="21" t="n">
+      <c r="A40" s="12" t="n">
         <v>24</v>
       </c>
-      <c r="B40" s="22" t="inlineStr">
+      <c r="B40" s="20" t="inlineStr">
         <is>
           <t>40.0%</t>
         </is>
       </c>
-      <c r="C40" s="25" t="n">
+      <c r="C40" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="D40" s="24" t="inlineStr">
+      <c r="D40" s="22" t="inlineStr">
         <is>
           <t>Reprobado (Insuficiente)</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="21" t="n">
+      <c r="A41" s="12" t="n">
         <v>23</v>
       </c>
-      <c r="B41" s="22" t="inlineStr">
+      <c r="B41" s="20" t="inlineStr">
         <is>
           <t>38.3%</t>
         </is>
       </c>
-      <c r="C41" s="25" t="n">
+      <c r="C41" s="23" t="n">
         <v>2.9</v>
       </c>
-      <c r="D41" s="24" t="inlineStr">
+      <c r="D41" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="21" t="n">
+      <c r="A42" s="12" t="n">
         <v>22</v>
       </c>
-      <c r="B42" s="22" t="inlineStr">
+      <c r="B42" s="20" t="inlineStr">
         <is>
           <t>36.7%</t>
         </is>
       </c>
-      <c r="C42" s="25" t="n">
+      <c r="C42" s="23" t="n">
         <v>2.8</v>
       </c>
-      <c r="D42" s="24" t="inlineStr">
+      <c r="D42" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="21" t="n">
+      <c r="A43" s="12" t="n">
         <v>21</v>
       </c>
-      <c r="B43" s="22" t="inlineStr">
+      <c r="B43" s="20" t="inlineStr">
         <is>
           <t>35.0%</t>
         </is>
       </c>
-      <c r="C43" s="25" t="n">
+      <c r="C43" s="23" t="n">
         <v>2.8</v>
       </c>
-      <c r="D43" s="24" t="inlineStr">
+      <c r="D43" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="21" t="n">
+      <c r="A44" s="12" t="n">
         <v>20</v>
       </c>
-      <c r="B44" s="22" t="inlineStr">
+      <c r="B44" s="20" t="inlineStr">
         <is>
           <t>33.3%</t>
         </is>
       </c>
-      <c r="C44" s="25" t="n">
+      <c r="C44" s="23" t="n">
         <v>2.7</v>
       </c>
-      <c r="D44" s="24" t="inlineStr">
+      <c r="D44" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="21" t="n">
+      <c r="A45" s="12" t="n">
         <v>19</v>
       </c>
-      <c r="B45" s="22" t="inlineStr">
+      <c r="B45" s="20" t="inlineStr">
         <is>
           <t>31.7%</t>
         </is>
       </c>
-      <c r="C45" s="25" t="n">
+      <c r="C45" s="23" t="n">
         <v>2.6</v>
       </c>
-      <c r="D45" s="24" t="inlineStr">
+      <c r="D45" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="21" t="n">
+      <c r="A46" s="12" t="n">
         <v>18</v>
       </c>
-      <c r="B46" s="22" t="inlineStr">
+      <c r="B46" s="20" t="inlineStr">
         <is>
           <t>30.0%</t>
         </is>
       </c>
-      <c r="C46" s="25" t="n">
+      <c r="C46" s="23" t="n">
         <v>2.5</v>
       </c>
-      <c r="D46" s="24" t="inlineStr">
+      <c r="D46" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="21" t="n">
+      <c r="A47" s="12" t="n">
         <v>17</v>
       </c>
-      <c r="B47" s="22" t="inlineStr">
+      <c r="B47" s="20" t="inlineStr">
         <is>
           <t>28.3%</t>
         </is>
       </c>
-      <c r="C47" s="25" t="n">
+      <c r="C47" s="23" t="n">
         <v>2.4</v>
       </c>
-      <c r="D47" s="24" t="inlineStr">
+      <c r="D47" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="21" t="n">
+      <c r="A48" s="12" t="n">
         <v>16</v>
       </c>
-      <c r="B48" s="22" t="inlineStr">
+      <c r="B48" s="20" t="inlineStr">
         <is>
           <t>26.7%</t>
         </is>
       </c>
-      <c r="C48" s="25" t="n">
+      <c r="C48" s="23" t="n">
         <v>2.3</v>
       </c>
-      <c r="D48" s="24" t="inlineStr">
+      <c r="D48" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="21" t="n">
+      <c r="A49" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="B49" s="22" t="inlineStr">
+      <c r="B49" s="20" t="inlineStr">
         <is>
           <t>25.0%</t>
         </is>
       </c>
-      <c r="C49" s="25" t="n">
+      <c r="C49" s="23" t="n">
         <v>2.2</v>
       </c>
-      <c r="D49" s="24" t="inlineStr">
+      <c r="D49" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="21" t="n">
+      <c r="A50" s="12" t="n">
         <v>14</v>
       </c>
-      <c r="B50" s="22" t="inlineStr">
+      <c r="B50" s="20" t="inlineStr">
         <is>
           <t>23.3%</t>
         </is>
       </c>
-      <c r="C50" s="25" t="n">
+      <c r="C50" s="23" t="n">
         <v>2.2</v>
       </c>
-      <c r="D50" s="24" t="inlineStr">
+      <c r="D50" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="21" t="n">
+      <c r="A51" s="12" t="n">
         <v>13</v>
       </c>
-      <c r="B51" s="22" t="inlineStr">
+      <c r="B51" s="20" t="inlineStr">
         <is>
           <t>21.7%</t>
         </is>
       </c>
-      <c r="C51" s="25" t="n">
+      <c r="C51" s="23" t="n">
         <v>2.1</v>
       </c>
-      <c r="D51" s="24" t="inlineStr">
+      <c r="D51" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="21" t="n">
+      <c r="A52" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="B52" s="22" t="inlineStr">
+      <c r="B52" s="20" t="inlineStr">
         <is>
           <t>20.0%</t>
         </is>
       </c>
-      <c r="C52" s="25" t="n">
+      <c r="C52" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="D52" s="24" t="inlineStr">
+      <c r="D52" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="21" t="n">
+      <c r="A53" s="12" t="n">
         <v>11</v>
       </c>
-      <c r="B53" s="22" t="inlineStr">
+      <c r="B53" s="20" t="inlineStr">
         <is>
           <t>18.3%</t>
         </is>
       </c>
-      <c r="C53" s="25" t="n">
+      <c r="C53" s="23" t="n">
         <v>1.9</v>
       </c>
-      <c r="D53" s="24" t="inlineStr">
+      <c r="D53" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="21" t="n">
+      <c r="A54" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="B54" s="22" t="inlineStr">
+      <c r="B54" s="20" t="inlineStr">
         <is>
           <t>16.7%</t>
         </is>
       </c>
-      <c r="C54" s="25" t="n">
+      <c r="C54" s="23" t="n">
         <v>1.8</v>
       </c>
-      <c r="D54" s="24" t="inlineStr">
+      <c r="D54" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="21" t="n">
+      <c r="A55" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="B55" s="22" t="inlineStr">
+      <c r="B55" s="20" t="inlineStr">
         <is>
           <t>15.0%</t>
         </is>
       </c>
-      <c r="C55" s="25" t="n">
+      <c r="C55" s="23" t="n">
         <v>1.8</v>
       </c>
-      <c r="D55" s="24" t="inlineStr">
+      <c r="D55" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
-      <c r="A56" s="21" t="n">
+      <c r="A56" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="B56" s="22" t="inlineStr">
+      <c r="B56" s="20" t="inlineStr">
         <is>
           <t>13.3%</t>
         </is>
       </c>
-      <c r="C56" s="25" t="n">
+      <c r="C56" s="23" t="n">
         <v>1.7</v>
       </c>
-      <c r="D56" s="24" t="inlineStr">
+      <c r="D56" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="21" t="n">
+      <c r="A57" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="B57" s="22" t="inlineStr">
+      <c r="B57" s="20" t="inlineStr">
         <is>
           <t>11.7%</t>
         </is>
       </c>
-      <c r="C57" s="25" t="n">
+      <c r="C57" s="23" t="n">
         <v>1.6</v>
       </c>
-      <c r="D57" s="24" t="inlineStr">
+      <c r="D57" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="21" t="n">
+      <c r="A58" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B58" s="22" t="inlineStr">
+      <c r="B58" s="20" t="inlineStr">
         <is>
           <t>10.0%</t>
         </is>
       </c>
-      <c r="C58" s="25" t="n">
+      <c r="C58" s="23" t="n">
         <v>1.5</v>
       </c>
-      <c r="D58" s="24" t="inlineStr">
+      <c r="D58" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="21" t="n">
+      <c r="A59" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="B59" s="22" t="inlineStr">
+      <c r="B59" s="20" t="inlineStr">
         <is>
           <t>8.3%</t>
         </is>
       </c>
-      <c r="C59" s="25" t="n">
+      <c r="C59" s="23" t="n">
         <v>1.4</v>
       </c>
-      <c r="D59" s="24" t="inlineStr">
+      <c r="D59" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="21" t="n">
+      <c r="A60" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B60" s="22" t="inlineStr">
+      <c r="B60" s="20" t="inlineStr">
         <is>
           <t>6.7%</t>
         </is>
       </c>
-      <c r="C60" s="25" t="n">
+      <c r="C60" s="23" t="n">
         <v>1.3</v>
       </c>
-      <c r="D60" s="24" t="inlineStr">
+      <c r="D60" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
-      <c r="A61" s="21" t="n">
+      <c r="A61" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B61" s="22" t="inlineStr">
+      <c r="B61" s="20" t="inlineStr">
         <is>
           <t>5.0%</t>
         </is>
       </c>
-      <c r="C61" s="25" t="n">
+      <c r="C61" s="23" t="n">
         <v>1.2</v>
       </c>
-      <c r="D61" s="24" t="inlineStr">
+      <c r="D61" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
-      <c r="A62" s="21" t="n">
+      <c r="A62" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B62" s="22" t="inlineStr">
+      <c r="B62" s="20" t="inlineStr">
         <is>
           <t>3.3%</t>
         </is>
       </c>
-      <c r="C62" s="25" t="n">
+      <c r="C62" s="23" t="n">
         <v>1.2</v>
       </c>
-      <c r="D62" s="24" t="inlineStr">
+      <c r="D62" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="63" ht="18" customHeight="1">
-      <c r="A63" s="21" t="n">
+      <c r="A63" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B63" s="22" t="inlineStr">
+      <c r="B63" s="20" t="inlineStr">
         <is>
           <t>1.7%</t>
         </is>
       </c>
-      <c r="C63" s="25" t="n">
+      <c r="C63" s="23" t="n">
         <v>1.1</v>
       </c>
-      <c r="D63" s="24" t="inlineStr">
+      <c r="D63" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>
       </c>
     </row>
     <row r="64" ht="18" customHeight="1">
-      <c r="A64" s="21" t="n">
+      <c r="A64" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="B64" s="22" t="inlineStr">
+      <c r="B64" s="20" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
-      <c r="C64" s="25" t="n">
+      <c r="C64" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D64" s="24" t="inlineStr">
+      <c r="D64" s="22" t="inlineStr">
         <is>
           <t>Deficiente / Sin Entrega</t>
         </is>

</xml_diff>